<commit_message>
feat: implement students backend slices 1 and 2
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02DE905-CA82-4A9E-A293-95CC88A2C8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TemplateDoHistorico - Model Nam" sheetId="1" r:id="rId4"/>
+    <sheet name="TemplateDoHistorico - Model Nam" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -30,15 +39,87 @@
   <si>
     <t>Observations</t>
   </si>
+  <si>
+    <t># Implementer Prompt - Iteration 01
+Implement only the first backend slice for student management.
+Project context:
+- Node + TypeScript backend
+- JSON persistence
+- current server already boots successfully
+- keep changes small and localized
+Required scope for this iteration:
+- create a modular student backend slice
+- implement GET /api/students
+- implement POST /api/students
+- persist students in a JSON file under the data directory
+- validate required fields: name, cpf, email
+- return clear HTTP responses for invalid input
+Constraints:
+- do not implement update or delete
+- do not touch frontend
+- do not implement classes, assessments, or notifications
+- do not refactor unrelated files
+- do not place all logic in route files
+Expected response format:
+1. Objective
+2. Files to change
+3. Out of scope
+4. Implementation summary
+5. Manual validation steps
+6. Risks or caveats</t>
+  </si>
+  <si>
+    <t>Accepted with manual adjustment</t>
+  </si>
+  <si>
+    <t>Useful for a small backend slice with clear scope, but still required close review for semantic quality and clean validation design.</t>
+  </si>
+  <si>
+    <t>The implementation worked functionally, but the validation layer initially had semantic issues in its error modeling. A payload-level validation error was modeled as a field-level error, and the validator also included an artificial fallback branch mainly for TypeScript narrowing rather than domain clarity. A small manual adjustment was necessary.</t>
+  </si>
+  <si>
+    <t>The agent respected the requested scope and produced a reasonably modular result with routing, validation, repository logic, and JSON persistence separated. Manual validation confirmed that GET and POST worked correctly and that invalid payloads were rejected. The main quality issue was not functionality, but the design of the validation response shape. This should be constrained more explicitly in future prompts.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 02
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-02/00-iteration-brief.md
+- sistema/docs/iterations/iteration-02/01-planner-output.md
+- sistema/server/src/routes/index.ts
+- sistema/server/src/modules/students/index.ts
+- sistema/server/src/modules/students/student.repository.ts
+- sistema/server/src/modules/students/student.validation.ts
+- sistema/server/src/shared/types/domain.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly, but the first validation attempt was temporarily confused by pre-existing duplicated records already present in students.json. The duplicate-check logic worked correctly on a clean dataset, but the iteration depended on cleaning legacy duplicated test data before update validation could be interpreted correctly.</t>
+  </si>
+  <si>
+    <t>Accepted</t>
+  </si>
+  <si>
+    <t>Good result for a medium-sized backend slice. The agent respected scope, improved modularity with a service layer, and implemented the required HTTP behaviors with less manual adjustment than in Iteration 01.</t>
+  </si>
+  <si>
+    <t>The agent handled this iteration better than the previous one because the prompt required planning first and explicitly encouraged a service layer when the module grew. Duplicate checks and update rules were centralized more cleanly. The main caveat was not code failure, but confusion caused by previously duplicated test records in the JSON file. Future prompts should continue to enforce thin routes, shared validation, and centralized conflict logic.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -50,19 +131,14 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <b/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="1"/>
+      <b/>
+      <i/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
@@ -246,54 +322,57 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+  <cellXfs count="16">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -304,28 +383,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ffa5a5a5"/>
-      <rgbColor rgb="ffbdc0bf"/>
-      <rgbColor rgb="ff3f3f3f"/>
-      <rgbColor rgb="ffdbdbdb"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="FFA5A5A5"/>
+      <rgbColor rgb="FFBDC0BF"/>
+      <rgbColor rgb="FF3F3F3F"/>
+      <rgbColor rgb="FFDBDBDB"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Blank">
   <a:themeElements>
     <a:clrScheme name="Blank">
       <a:dk1>
@@ -527,7 +663,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -545,7 +681,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -574,7 +710,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -599,7 +735,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -624,7 +760,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -649,7 +785,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -674,7 +810,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -699,7 +835,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -724,7 +860,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -749,7 +885,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -774,7 +910,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -787,9 +923,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -806,7 +948,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -824,7 +966,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -849,7 +991,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -874,7 +1016,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -899,7 +1041,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -924,7 +1066,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -949,7 +1091,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -974,7 +1116,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -999,7 +1141,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1024,7 +1166,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1049,7 +1191,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1062,9 +1204,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1078,7 +1226,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1096,7 +1244,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1125,7 +1273,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1150,7 +1298,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1175,7 +1323,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1200,7 +1348,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1225,7 +1373,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1250,7 +1398,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1275,7 +1423,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1300,7 +1448,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1325,7 +1473,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1338,489 +1486,517 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E63"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="44.3516" style="1" customWidth="1"/>
-    <col min="2" max="4" width="16.3516" style="1" customWidth="1"/>
-    <col min="5" max="5" width="31.5" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col min="1" max="1" width="44.28515625" style="1" customWidth="1"/>
+    <col min="2" max="4" width="16.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="16.28515625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.65" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:5" ht="27.6" customHeight="1">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
-    </row>
-    <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" t="s" s="5">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="14"/>
+    </row>
+    <row r="2" spans="1:5" ht="20.25" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s" s="6">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s" s="6">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s" s="6">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" t="s" s="6">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-    </row>
-    <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-    </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-    </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-    </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-    </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-    </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-    </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-    </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-    </row>
-    <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-    </row>
-    <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-    </row>
-    <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-    </row>
-    <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-    </row>
-    <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="10"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-    </row>
-    <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="10"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-    </row>
-    <row r="23" ht="20.05" customHeight="1">
-      <c r="A23" s="13"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-    </row>
-    <row r="24" ht="20.05" customHeight="1">
-      <c r="A24" s="10"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-    </row>
-    <row r="25" ht="20.05" customHeight="1">
-      <c r="A25" s="10"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-    </row>
-    <row r="26" ht="20.05" customHeight="1">
-      <c r="A26" s="10"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-    </row>
-    <row r="27" ht="20.05" customHeight="1">
-      <c r="A27" s="10"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-    </row>
-    <row r="28" ht="20.05" customHeight="1">
-      <c r="A28" s="10"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-    </row>
-    <row r="29" ht="20.05" customHeight="1">
-      <c r="A29" s="10"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-    </row>
-    <row r="30" ht="20.05" customHeight="1">
-      <c r="A30" s="10"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-    </row>
-    <row r="31" ht="20.05" customHeight="1">
-      <c r="A31" s="10"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-    </row>
-    <row r="32" ht="20.05" customHeight="1">
-      <c r="A32" s="10"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-    </row>
-    <row r="33" ht="20.05" customHeight="1">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-    </row>
-    <row r="34" ht="20.05" customHeight="1">
-      <c r="A34" s="10"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-    </row>
-    <row r="35" ht="20.05" customHeight="1">
-      <c r="A35" s="10"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-    </row>
-    <row r="36" ht="20.05" customHeight="1">
-      <c r="A36" s="10"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-    </row>
-    <row r="37" ht="20.05" customHeight="1">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-    </row>
-    <row r="38" ht="20.05" customHeight="1">
-      <c r="A38" s="10"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-    </row>
-    <row r="39" ht="20.05" customHeight="1">
-      <c r="A39" s="10"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-    </row>
-    <row r="40" ht="20.05" customHeight="1">
-      <c r="A40" s="10"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-    </row>
-    <row r="41" ht="20.05" customHeight="1">
-      <c r="A41" s="10"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-    </row>
-    <row r="42" ht="20.05" customHeight="1">
-      <c r="A42" s="10"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-    </row>
-    <row r="43" ht="20.05" customHeight="1">
-      <c r="A43" s="10"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-    </row>
-    <row r="44" ht="20.05" customHeight="1">
-      <c r="A44" s="10"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-    </row>
-    <row r="45" ht="20.05" customHeight="1">
-      <c r="A45" s="13"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-    </row>
-    <row r="46" ht="20.05" customHeight="1">
-      <c r="A46" s="13"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-    </row>
-    <row r="47" ht="20.05" customHeight="1">
-      <c r="A47" s="13"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-    </row>
-    <row r="48" ht="20.05" customHeight="1">
-      <c r="A48" s="13"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-    </row>
-    <row r="49" ht="20.05" customHeight="1">
-      <c r="A49" s="13"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="12"/>
-    </row>
-    <row r="50" ht="20.05" customHeight="1">
-      <c r="A50" s="13"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="12"/>
-    </row>
-    <row r="51" ht="20.05" customHeight="1">
-      <c r="A51" s="13"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="12"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="12"/>
-    </row>
-    <row r="52" ht="20.05" customHeight="1">
-      <c r="A52" s="13"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="12"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="12"/>
-    </row>
-    <row r="53" ht="20.05" customHeight="1">
-      <c r="A53" s="13"/>
-      <c r="B53" s="11"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="12"/>
-    </row>
-    <row r="54" ht="20.05" customHeight="1">
-      <c r="A54" s="13"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="12"/>
-    </row>
-    <row r="55" ht="20.05" customHeight="1">
-      <c r="A55" s="13"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="12"/>
-      <c r="E55" s="12"/>
-    </row>
-    <row r="56" ht="20.05" customHeight="1">
-      <c r="A56" s="13"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="12"/>
-      <c r="D56" s="12"/>
-      <c r="E56" s="12"/>
-    </row>
-    <row r="57" ht="20.05" customHeight="1">
-      <c r="A57" s="13"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="12"/>
-    </row>
-    <row r="58" ht="20.05" customHeight="1">
-      <c r="A58" s="13"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="12"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="12"/>
-    </row>
-    <row r="59" ht="20.05" customHeight="1">
-      <c r="A59" s="13"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
-    </row>
-    <row r="60" ht="20.05" customHeight="1">
-      <c r="A60" s="13"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="12"/>
-      <c r="D60" s="12"/>
-      <c r="E60" s="12"/>
-    </row>
-    <row r="61" ht="20.05" customHeight="1">
-      <c r="A61" s="13"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="12"/>
-      <c r="D61" s="12"/>
-      <c r="E61" s="12"/>
-    </row>
-    <row r="62" ht="20.05" customHeight="1">
-      <c r="A62" s="13"/>
-      <c r="B62" s="11"/>
-      <c r="C62" s="12"/>
-      <c r="D62" s="12"/>
-      <c r="E62" s="12"/>
-    </row>
-    <row r="63" ht="20.05" customHeight="1">
-      <c r="A63" s="13"/>
-      <c r="B63" s="11"/>
-      <c r="C63" s="12"/>
-      <c r="D63" s="12"/>
-      <c r="E63" s="12"/>
+    <row r="3" spans="1:5" ht="20.25" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A5" s="15"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+    </row>
+    <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A6" s="7"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+    </row>
+    <row r="7" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A7" s="7"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+    </row>
+    <row r="8" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+    </row>
+    <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A9" s="7"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+    </row>
+    <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A10" s="7"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+    </row>
+    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+    </row>
+    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A16" s="7"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+    </row>
+    <row r="17" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A17" s="7"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A18" s="7"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A19" s="7"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+    </row>
+    <row r="20" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A20" s="7"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+    </row>
+    <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A21" s="7"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A22" s="7"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+    </row>
+    <row r="23" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A23" s="10"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+    </row>
+    <row r="24" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A24" s="7"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+    </row>
+    <row r="25" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A25" s="7"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+    </row>
+    <row r="26" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A26" s="7"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+    </row>
+    <row r="27" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A27" s="7"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+    </row>
+    <row r="28" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A28" s="7"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+    </row>
+    <row r="29" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A29" s="7"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+    </row>
+    <row r="30" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A30" s="7"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+    </row>
+    <row r="31" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A31" s="7"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+    </row>
+    <row r="32" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+    </row>
+    <row r="33" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A33" s="7"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+    </row>
+    <row r="34" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A34" s="7"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+    </row>
+    <row r="35" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A35" s="7"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+    </row>
+    <row r="36" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A36" s="7"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+    </row>
+    <row r="37" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A37" s="7"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+    </row>
+    <row r="38" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A38" s="7"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+    </row>
+    <row r="39" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A39" s="7"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+    </row>
+    <row r="40" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A40" s="7"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+    </row>
+    <row r="41" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A41" s="7"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+    </row>
+    <row r="42" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A42" s="7"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+    </row>
+    <row r="43" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A43" s="7"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+    </row>
+    <row r="44" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A44" s="7"/>
+      <c r="B44" s="11"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+    </row>
+    <row r="45" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A45" s="10"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+    </row>
+    <row r="46" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A46" s="10"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+    </row>
+    <row r="47" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A47" s="10"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+    </row>
+    <row r="48" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A48" s="10"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+    </row>
+    <row r="49" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A49" s="10"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+    </row>
+    <row r="50" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A50" s="10"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+    </row>
+    <row r="51" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A51" s="10"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+    </row>
+    <row r="52" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A52" s="10"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+    </row>
+    <row r="53" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A53" s="10"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+    </row>
+    <row r="54" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A54" s="10"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+    </row>
+    <row r="55" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A55" s="10"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+    </row>
+    <row r="56" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A56" s="10"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+    </row>
+    <row r="57" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A57" s="10"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+    </row>
+    <row r="58" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A58" s="10"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
+    </row>
+    <row r="59" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A59" s="10"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+    </row>
+    <row r="60" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A60" s="10"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+    </row>
+    <row r="61" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A61" s="10"/>
+      <c r="B61" s="8"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+    </row>
+    <row r="62" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A62" s="10"/>
+      <c r="B62" s="8"/>
+      <c r="C62" s="9"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="9"/>
+    </row>
+    <row r="63" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A63" s="10"/>
+      <c r="B63" s="8"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
feat: add students delete endpoint
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02DE905-CA82-4A9E-A293-95CC88A2C8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8856427B-8F60-4203-A15E-32B28E08D019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -113,6 +113,38 @@
   </si>
   <si>
     <t>The agent handled this iteration better than the previous one because the prompt required planning first and explicitly encouraged a service layer when the module grew. Duplicate checks and update rules were centralized more cleanly. The main caveat was not code failure, but confusion caused by previously duplicated test records in the JSON file. Future prompts should continue to enforce thin routes, shared validation, and centralized conflict logic.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 03
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-03/00-iteration-brief.md
+- sistema/docs/iterations/iteration-03/01-planner-output.md
+- sistema/server/src/routes/index.ts
+- sistema/server/src/modules/students/index.ts
+- sistema/server/src/modules/students/student.repository.ts
+- sistema/server/src/modules/students/student.service.ts
+- sistema/server/src/modules/students/student.validation.ts
+- sistema/server/src/shared/types/domain.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and required no meaningful manual code correction after generation. The main remaining concerns are architectural rather than functional: repository path handling still relies on process.cwd(), and JSON-file persistence remains simple and non-transactional.</t>
+  </si>
+  <si>
+    <t>Good result for a focused backend slice. The agent respected the scope, preserved modularity, and extended the students backend cleanly without introducing unnecessary changes.</t>
+  </si>
+  <si>
+    <t>This iteration went more smoothly than the earlier ones because the prompt constrained the change set tightly and the students module already had a service/repository structure to extend. The delete behavior was implemented cleanly with correct status codes and correct persistence updates. The next prompts should continue using the same discipline of thin routes and localized changes.</t>
   </si>
 </sst>
 </file>
@@ -1579,14 +1611,24 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A5" s="15"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
+      <c r="A5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A6" s="7"/>
+      <c r="A6" s="15"/>
       <c r="B6" s="8"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>

</xml_diff>

<commit_message>
test: add students backend acceptance scenarios
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8856427B-8F60-4203-A15E-32B28E08D019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4617F97-037E-4FE3-9AC5-34264DA28C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -145,6 +145,37 @@
   </si>
   <si>
     <t>This iteration went more smoothly than the earlier ones because the prompt constrained the change set tightly and the students module already had a service/repository structure to extend. The delete behavior was implemented cleanly with correct status codes and correct persistence updates. The next prompts should continue using the same discipline of thin routes and localized changes.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 04
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-04/00-iteration-brief.md
+- sistema/docs/iterations/iteration-04/01-planner-output.md
+- sistema/server/package.json
+- sistema/server/src/modules/students/index.ts
+- sistema/server/src/modules/students/student.service.ts
+- sistema/server/src/modules/students/student.repository.ts
+- sistema/server/data/students.json
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and did not require backend business-logic changes, but the test layer depends on a separately running local API and still inherits the simplicity of JSON-file state management. The suite also emits a Node-version warning in this environment, although execution succeeds.</t>
+  </si>
+  <si>
+    <t>Good result for a test-infrastructure iteration. The agent respected scope, kept the setup simple, and created readable acceptance scenarios with a practical reset strategy.</t>
+  </si>
+  <si>
+    <t>This iteration was successful because the prompts constrained the solution to minimal Cucumber infrastructure and discouraged unnecessary complexity. The use of JavaScript step definitions and deterministic reset hooks kept the setup understandable. The main lesson is that stable acceptance tests for JSON-backed systems require explicit state control.</t>
   </si>
 </sst>
 </file>
@@ -358,7 +389,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -403,9 +434,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1628,11 +1656,21 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A6" s="15"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
+      <c r="A6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="7" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="7"/>

</xml_diff>

<commit_message>
fix: harden students frontend cpf input and list layout
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4617F97-037E-4FE3-9AC5-34264DA28C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA92C5D-4EAD-4BA8-89FC-6A017FD56A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -176,6 +176,66 @@
   </si>
   <si>
     <t>This iteration was successful because the prompts constrained the solution to minimal Cucumber infrastructure and discouraged unnecessary complexity. The use of JavaScript step definitions and deterministic reset hooks kept the setup understandable. The main lesson is that stable acceptance tests for JSON-backed systems require explicit state control.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 05
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-05/00-iteration-brief.md
+- sistema/docs/iterations/iteration-05/01-planner-output.md
+- sistema/client/src/pages/StudentsPage.tsx
+- sistema/client/src/config/api.ts
+- sistema/client/src/types/domain.ts
+- sistema/client/src/router.tsx
+- sistema/client/src/styles.css
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The first students frontend slice worked well and looked good, but manual review found two follow-up UX issues: long student values could still stress the list layout, and CPF input was still too permissive in the UI. These issues are better handled in a dedicated corrective frontend-hardening iteration.</t>
+  </si>
+  <si>
+    <t>Good result for a first frontend slice. The agent delivered a clearly improved and functional students page with clean visual organization, but a small corrective pass is still needed for stronger UX resilience.</t>
+  </si>
+  <si>
+    <t>The agent handled the visual requirement reasonably well once the prompt explicitly required a polished result. The best outcome came from combining functional scope with aesthetic constraints in the prompt. Manual review remains essential because overflow and input-hardening issues were only visible after real interaction with the page.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 06
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-06/00-iteration-brief.md
+- sistema/docs/iterations/iteration-06/01-planner-output.md
+- sistema/client/src/pages/StudentsPage.tsx
+- sistema/client/src/config/studentsApi.ts
+- sistema/client/src/styles.css
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and solved the immediate frontend UX issues, but CPF validation is still enforced only in the frontend. This means invalid CPF values could still be sent directly to the backend API outside the UI, so a backend hardening follow-up is still necessary.</t>
+  </si>
+  <si>
+    <t>Good corrective iteration. The agent stayed scoped, preserved the visual quality of the page, and resolved the manual-review UX issues without overengineering the solution.</t>
+  </si>
+  <si>
+    <t>This iteration worked well because the prompt was tightly constrained around two concrete review findings: input hardening and layout resilience. The combination of simple input sanitization and targeted CSS was enough to fix the visible problems quickly. The next important step is to align backend validation with the improved frontend behavior.</t>
   </si>
 </sst>
 </file>
@@ -1673,18 +1733,38 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
+      <c r="A7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="8" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
+      <c r="A8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="7"/>

</xml_diff>

<commit_message>
fix: harden backend cpf validation for students
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA92C5D-4EAD-4BA8-89FC-6A017FD56A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D146269-09AE-4A84-9FAE-76A8B8C87432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -236,6 +236,35 @@
   </si>
   <si>
     <t>This iteration worked well because the prompt was tightly constrained around two concrete review findings: input hardening and layout resilience. The combination of simple input sanitization and targeted CSS was enough to fix the visible problems quickly. The next important step is to align backend validation with the improved frontend behavior.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 07
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-07/00-iteration-brief.md
+- sistema/docs/iterations/iteration-07/01-planner-output.md
+- sistema/server/src/modules/students/student.validation.ts
+- sistema/server/src/modules/students/student.service.ts
+- sistema/server/src/modules/students/index.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and kept the rule centralized, but CPF validation is still intentionally basic. It now enforces numeric-only plus exact length 11, but it does not attempt richer CPF business validation beyond that scope.</t>
+  </si>
+  <si>
+    <t>Good backend hardening iteration. The agent stayed narrowly scoped, changed only the right layer, and aligned backend validation with the frontend behavior without unnecessary refactoring.</t>
+  </si>
+  <si>
+    <t>This iteration worked well because the requirement was simple, explicit, and strongly constrained toward one shared validation point. The result improved system integrity by ensuring invalid CPF values can no longer bypass the frontend and enter through direct API calls.</t>
   </si>
 </sst>
 </file>
@@ -1767,11 +1796,21 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
+      <c r="A9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="7"/>

</xml_diff>

<commit_message>
feat: add students edit mode in frontend
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D146269-09AE-4A84-9FAE-76A8B8C87432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6602332A-EA6C-4175-A600-5BD0E6C9BFA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TemplateDoHistorico - Model Nam" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -265,6 +265,36 @@
   </si>
   <si>
     <t>This iteration worked well because the requirement was simple, explicit, and strongly constrained toward one shared validation point. The result improved system integrity by ensuring invalid CPF values can no longer bypass the frontend and enter through direct API calls.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 08
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-08/00-iteration-brief.md
+- sistema/docs/iterations/iteration-08/01-planner-output.md
+- sistema/client/src/pages/StudentsPage.tsx
+- sistema/client/src/config/studentsApi.ts
+- sistema/client/src/styles.css
+- sistema/client/src/types/domain.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and delivered edit mode cleanly, but the students page is becoming more feature-dense. The current shared form approach still works well, yet future iterations should keep guarding against excessive logic growth inside the page component.</t>
+  </si>
+  <si>
+    <t>Good frontend iteration. The agent stayed scoped, preserved the current visual quality, and added edit mode without breaking the existing create flow.</t>
+  </si>
+  <si>
+    <t>This iteration worked well because the prompt explicitly required reuse of the existing form and strong visual edit-mode cues. That prevented unnecessary duplication and kept the page coherent. The next step should complete the students frontend flow with delete functionality.</t>
   </si>
 </sst>
 </file>
@@ -1658,16 +1688,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E63"/>
-  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.26953125" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="44.28515625" style="1" customWidth="1"/>
-    <col min="2" max="4" width="16.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="31.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="16.28515625" style="1"/>
+    <col min="1" max="1" width="44.26953125" style="1" customWidth="1"/>
+    <col min="2" max="4" width="16.26953125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="16.26953125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.6" customHeight="1">
+    <row r="1" spans="1:5" ht="27.65" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1710,7 +1740,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="4" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
@@ -1727,7 +1757,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="5" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -1744,7 +1774,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="6" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>20</v>
       </c>
@@ -1761,7 +1791,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="7" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>24</v>
       </c>
@@ -1778,7 +1808,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="8" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>28</v>
       </c>
@@ -1795,7 +1825,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="9" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>32</v>
       </c>
@@ -1812,378 +1842,388 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-    </row>
-    <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="10" spans="1:5" ht="20.149999999999999" customHeight="1">
+      <c r="A10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A11" s="7"/>
       <c r="B11" s="8"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
     </row>
-    <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="12" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A12" s="7"/>
       <c r="B12" s="8"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
     </row>
-    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="13" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="14" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
     </row>
-    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="15" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
     </row>
-    <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="16" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="17" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
     </row>
-    <row r="18" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="18" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
     </row>
-    <row r="19" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="19" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A19" s="7"/>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
     </row>
-    <row r="20" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="20" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A20" s="7"/>
       <c r="B20" s="8"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
     </row>
-    <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="21" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A21" s="7"/>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
     </row>
-    <row r="22" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="22" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="8"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
     </row>
-    <row r="23" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="23" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A23" s="10"/>
       <c r="B23" s="8"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
     </row>
-    <row r="24" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="24" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A24" s="7"/>
       <c r="B24" s="8"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
     </row>
-    <row r="25" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="25" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A25" s="7"/>
       <c r="B25" s="8"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
     </row>
-    <row r="26" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="26" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A26" s="7"/>
       <c r="B26" s="8"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
     </row>
-    <row r="27" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="27" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A27" s="7"/>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
     </row>
-    <row r="28" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="28" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A28" s="7"/>
       <c r="B28" s="8"/>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
     </row>
-    <row r="29" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="29" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A29" s="7"/>
       <c r="B29" s="8"/>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
     </row>
-    <row r="30" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="30" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A30" s="7"/>
       <c r="B30" s="8"/>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
     </row>
-    <row r="31" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="31" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A31" s="7"/>
       <c r="B31" s="8"/>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
     </row>
-    <row r="32" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="32" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A32" s="7"/>
       <c r="B32" s="8"/>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
     </row>
-    <row r="33" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="33" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A33" s="7"/>
       <c r="B33" s="8"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="34" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A34" s="7"/>
       <c r="B34" s="8"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
     </row>
-    <row r="35" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="35" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A35" s="7"/>
       <c r="B35" s="8"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
     </row>
-    <row r="36" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="36" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A36" s="7"/>
       <c r="B36" s="8"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
     </row>
-    <row r="37" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="37" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A37" s="7"/>
       <c r="B37" s="8"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="38" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A38" s="7"/>
       <c r="B38" s="8"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
     </row>
-    <row r="39" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="39" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A39" s="7"/>
       <c r="B39" s="8"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
     </row>
-    <row r="40" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="40" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A40" s="7"/>
       <c r="B40" s="8"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
     </row>
-    <row r="41" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="41" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A41" s="7"/>
       <c r="B41" s="8"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="42" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A42" s="7"/>
       <c r="B42" s="8"/>
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
     </row>
-    <row r="43" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="43" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A43" s="7"/>
       <c r="B43" s="8"/>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
     </row>
-    <row r="44" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="44" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A44" s="7"/>
       <c r="B44" s="11"/>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
     </row>
-    <row r="45" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="45" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A45" s="10"/>
       <c r="B45" s="8"/>
       <c r="C45" s="9"/>
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
     </row>
-    <row r="46" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="46" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A46" s="10"/>
       <c r="B46" s="8"/>
       <c r="C46" s="9"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
     </row>
-    <row r="47" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="47" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A47" s="10"/>
       <c r="B47" s="8"/>
       <c r="C47" s="9"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
     </row>
-    <row r="48" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="48" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A48" s="10"/>
       <c r="B48" s="8"/>
       <c r="C48" s="9"/>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
     </row>
-    <row r="49" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="49" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A49" s="10"/>
       <c r="B49" s="8"/>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
     </row>
-    <row r="50" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="50" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A50" s="10"/>
       <c r="B50" s="8"/>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
     </row>
-    <row r="51" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="51" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A51" s="10"/>
       <c r="B51" s="8"/>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
     </row>
-    <row r="52" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="52" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A52" s="10"/>
       <c r="B52" s="8"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
     </row>
-    <row r="53" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="53" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A53" s="10"/>
       <c r="B53" s="8"/>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
     </row>
-    <row r="54" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="54" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A54" s="10"/>
       <c r="B54" s="8"/>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
     </row>
-    <row r="55" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="55" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A55" s="10"/>
       <c r="B55" s="8"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
     </row>
-    <row r="56" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="56" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A56" s="10"/>
       <c r="B56" s="8"/>
       <c r="C56" s="9"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
     </row>
-    <row r="57" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="57" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A57" s="10"/>
       <c r="B57" s="8"/>
       <c r="C57" s="9"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
     </row>
-    <row r="58" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="58" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A58" s="10"/>
       <c r="B58" s="8"/>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
     </row>
-    <row r="59" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="59" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A59" s="10"/>
       <c r="B59" s="8"/>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
     </row>
-    <row r="60" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="60" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A60" s="10"/>
       <c r="B60" s="8"/>
       <c r="C60" s="9"/>
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
     </row>
-    <row r="61" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="61" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A61" s="10"/>
       <c r="B61" s="8"/>
       <c r="C61" s="9"/>
       <c r="D61" s="9"/>
       <c r="E61" s="9"/>
     </row>
-    <row r="62" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="62" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A62" s="10"/>
       <c r="B62" s="8"/>
       <c r="C62" s="9"/>
       <c r="D62" s="9"/>
       <c r="E62" s="9"/>
     </row>
-    <row r="63" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="63" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A63" s="10"/>
       <c r="B63" s="8"/>
       <c r="C63" s="9"/>

</xml_diff>

<commit_message>
feat: add students delete action in frontend
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6602332A-EA6C-4175-A600-5BD0E6C9BFA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEF7D06-2044-4003-9533-2AD569AB6ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -295,6 +295,36 @@
   </si>
   <si>
     <t>This iteration worked well because the prompt explicitly required reuse of the existing form and strong visual edit-mode cues. That prevented unnecessary duplication and kept the page coherent. The next step should complete the students frontend flow with delete functionality.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 09
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-09/00-iteration-brief.md
+- sistema/docs/iterations/iteration-09/01-planner-output.md
+- sistema/client/src/pages/StudentsPage.tsx
+- sistema/client/src/config/studentsApi.ts
+- sistema/client/src/styles.css
+- sistema/client/src/types/domain.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and kept the delete flow well scoped, but the students page now carries create, edit, and delete behavior in one component. The current localized approach still works, yet future iterations should continue watching for excessive UI-state growth.</t>
+  </si>
+  <si>
+    <t>Good frontend iteration. The agent preserved the current visual style, added delete cleanly, and kept the full students flow coherent without unnecessary complexity.</t>
+  </si>
+  <si>
+    <t>This iteration worked well because the prompt explicitly separated delete from confirmation-modal complexity and required correct interaction with edit mode. The result completed the core students frontend workflow while keeping the page visually consistent.</t>
   </si>
 </sst>
 </file>
@@ -1860,11 +1890,21 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="20.149999999999999" customHeight="1">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
+      <c r="A11" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="12" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A12" s="7"/>

</xml_diff>

<commit_message>
feat: add classes backend list and create flow
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEF7D06-2044-4003-9533-2AD569AB6ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C61E39-562D-40C6-83B1-2BD4E32E8CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TemplateDoHistorico - Model Nam" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -325,6 +325,36 @@
   </si>
   <si>
     <t>This iteration worked well because the prompt explicitly separated delete from confirmation-modal complexity and required correct interaction with edit mode. The result completed the core students frontend workflow while keeping the page visually consistent.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 10
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-10/00-iteration-brief.md
+- sistema/docs/iterations/iteration-10/01-planner-output.md
+- sistema/server/src/modules/classes/index.ts
+- sistema/server/src/routes/index.ts
+- sistema/server/src/shared/types/domain.ts
+- sistema/server/data/README.md
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and used the required class shape, but the classes backend is still intentionally basic. It covers only list/create plus payload validation and does not yet include update/delete, enrollment workflows, or assessment logic.</t>
+  </si>
+  <si>
+    <t>Good backend iteration. The agent stayed scoped, followed the modular pattern already established in students, and introduced the classes slice cleanly without drifting into broader functionality.</t>
+  </si>
+  <si>
+    <t>This iteration worked well because the required class shape and scope boundaries were stated very explicitly. That prevented field-name drift and helped keep the implementation localized. The next step should complete the classes backend with update/delete and then move toward class-related frontend flows.</t>
   </si>
 </sst>
 </file>
@@ -1718,16 +1748,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E63"/>
-  <sheetFormatPr defaultColWidth="16.26953125" defaultRowHeight="19.899999999999999" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="44.26953125" style="1" customWidth="1"/>
-    <col min="2" max="4" width="16.26953125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="31.453125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.26953125" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="16.26953125" style="1"/>
+    <col min="1" max="1" width="44.28515625" style="1" customWidth="1"/>
+    <col min="2" max="4" width="16.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="16.28515625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.65" customHeight="1">
+    <row r="1" spans="1:5" ht="27.6" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1770,7 +1800,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
@@ -1787,7 +1817,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -1804,7 +1834,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>20</v>
       </c>
@@ -1821,7 +1851,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="7" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>24</v>
       </c>
@@ -1838,7 +1868,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="8" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>28</v>
       </c>
@@ -1855,7 +1885,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>32</v>
       </c>
@@ -1872,7 +1902,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="7" t="s">
         <v>36</v>
       </c>
@@ -1889,7 +1919,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="7" t="s">
         <v>40</v>
       </c>
@@ -1906,364 +1936,374 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="20.149999999999999" customHeight="1">
-      <c r="A12" s="7"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-    </row>
-    <row r="13" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1">
+      <c r="A12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
     </row>
-    <row r="15" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
     </row>
-    <row r="16" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="17" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
     </row>
-    <row r="18" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="18" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
     </row>
-    <row r="19" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="19" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A19" s="7"/>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
     </row>
-    <row r="20" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="20" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A20" s="7"/>
       <c r="B20" s="8"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
     </row>
-    <row r="21" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A21" s="7"/>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
     </row>
-    <row r="22" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="22" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="8"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
     </row>
-    <row r="23" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="23" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="10"/>
       <c r="B23" s="8"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
     </row>
-    <row r="24" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="24" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A24" s="7"/>
       <c r="B24" s="8"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
     </row>
-    <row r="25" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="25" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A25" s="7"/>
       <c r="B25" s="8"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
     </row>
-    <row r="26" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="26" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A26" s="7"/>
       <c r="B26" s="8"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
     </row>
-    <row r="27" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="27" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="7"/>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
     </row>
-    <row r="28" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="28" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="7"/>
       <c r="B28" s="8"/>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
     </row>
-    <row r="29" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="29" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A29" s="7"/>
       <c r="B29" s="8"/>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
     </row>
-    <row r="30" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="30" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A30" s="7"/>
       <c r="B30" s="8"/>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
     </row>
-    <row r="31" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="31" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A31" s="7"/>
       <c r="B31" s="8"/>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
     </row>
-    <row r="32" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="32" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A32" s="7"/>
       <c r="B32" s="8"/>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
     </row>
-    <row r="33" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="33" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="7"/>
       <c r="B33" s="8"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="34" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="7"/>
       <c r="B34" s="8"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
     </row>
-    <row r="35" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="35" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="7"/>
       <c r="B35" s="8"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
     </row>
-    <row r="36" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="36" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="7"/>
       <c r="B36" s="8"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
     </row>
-    <row r="37" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="37" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="7"/>
       <c r="B37" s="8"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="38" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="7"/>
       <c r="B38" s="8"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
     </row>
-    <row r="39" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="39" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="7"/>
       <c r="B39" s="8"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
     </row>
-    <row r="40" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="40" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="7"/>
       <c r="B40" s="8"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
     </row>
-    <row r="41" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="41" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="7"/>
       <c r="B41" s="8"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="42" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="7"/>
       <c r="B42" s="8"/>
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
     </row>
-    <row r="43" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="43" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A43" s="7"/>
       <c r="B43" s="8"/>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
     </row>
-    <row r="44" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="44" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A44" s="7"/>
       <c r="B44" s="11"/>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
     </row>
-    <row r="45" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="45" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A45" s="10"/>
       <c r="B45" s="8"/>
       <c r="C45" s="9"/>
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
     </row>
-    <row r="46" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="46" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A46" s="10"/>
       <c r="B46" s="8"/>
       <c r="C46" s="9"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
     </row>
-    <row r="47" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="47" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A47" s="10"/>
       <c r="B47" s="8"/>
       <c r="C47" s="9"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
     </row>
-    <row r="48" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="48" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A48" s="10"/>
       <c r="B48" s="8"/>
       <c r="C48" s="9"/>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
     </row>
-    <row r="49" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="49" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A49" s="10"/>
       <c r="B49" s="8"/>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
     </row>
-    <row r="50" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="50" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A50" s="10"/>
       <c r="B50" s="8"/>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
     </row>
-    <row r="51" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="51" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A51" s="10"/>
       <c r="B51" s="8"/>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
     </row>
-    <row r="52" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="52" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A52" s="10"/>
       <c r="B52" s="8"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
     </row>
-    <row r="53" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="53" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A53" s="10"/>
       <c r="B53" s="8"/>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
     </row>
-    <row r="54" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="54" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A54" s="10"/>
       <c r="B54" s="8"/>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
     </row>
-    <row r="55" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="55" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="10"/>
       <c r="B55" s="8"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
     </row>
-    <row r="56" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="56" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A56" s="10"/>
       <c r="B56" s="8"/>
       <c r="C56" s="9"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
     </row>
-    <row r="57" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="57" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A57" s="10"/>
       <c r="B57" s="8"/>
       <c r="C57" s="9"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
     </row>
-    <row r="58" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="58" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A58" s="10"/>
       <c r="B58" s="8"/>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
     </row>
-    <row r="59" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="59" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A59" s="10"/>
       <c r="B59" s="8"/>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
     </row>
-    <row r="60" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="60" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A60" s="10"/>
       <c r="B60" s="8"/>
       <c r="C60" s="9"/>
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
     </row>
-    <row r="61" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="61" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A61" s="10"/>
       <c r="B61" s="8"/>
       <c r="C61" s="9"/>
       <c r="D61" s="9"/>
       <c r="E61" s="9"/>
     </row>
-    <row r="62" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="62" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A62" s="10"/>
       <c r="B62" s="8"/>
       <c r="C62" s="9"/>
       <c r="D62" s="9"/>
       <c r="E62" s="9"/>
     </row>
-    <row r="63" spans="1:5" ht="20.149999999999999" customHeight="1">
+    <row r="63" spans="1:5" ht="20.100000000000001" customHeight="1">
       <c r="A63" s="10"/>
       <c r="B63" s="8"/>
       <c r="C63" s="9"/>

</xml_diff>

<commit_message>
feat: add classes update and delete backend flow
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CC_UFPE\second-experiment-agents\second-experiment-agentic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C61E39-562D-40C6-83B1-2BD4E32E8CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF109BB-6D17-4463-B0B2-DE7C50957A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TemplateDoHistorico - Model Nam" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="52">
   <si>
     <t>Model Name and Version - Agent Name - Skills and Agents</t>
   </si>
@@ -355,6 +355,38 @@
   </si>
   <si>
     <t>This iteration worked well because the required class shape and scope boundaries were stated very explicitly. That prevented field-name drift and helped keep the implementation localized. The next step should complete the classes backend with update/delete and then move toward class-related frontend flows.</t>
+  </si>
+  <si>
+    <t># Implementer Prompt - Iteration 11
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-11/00-iteration-brief.md
+- sistema/docs/iterations/iteration-11/01-planner-output.md
+- sistema/server/src/modules/classes/index.ts
+- sistema/server/src/modules/classes/class.validation.ts
+- sistema/server/src/modules/classes/class.repository.ts
+- sistema/server/src/modules/classes/class.service.ts
+- sistema/server/src/shared/types/domain.ts
+- sistema/server/data/classes.json
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</t>
+  </si>
+  <si>
+    <t>The implementation behaved correctly and completed the basic classes backend CRUD, but update still uses full replacement semantics and persistence remains simple JSON file I/O. During manual validation, delete required a clean server restart, which appears to have been a local runtime refresh issue rather than a code bug.</t>
+  </si>
+  <si>
+    <t>Good backend iteration. The agent stayed scoped, completed the missing CRUD operations cleanly, and preserved the modular structure of the classes module.</t>
+  </si>
+  <si>
+    <t>This iteration worked well because the scope was tightly limited to update/delete and required consistent 404 handling. Reusing the existing validator helped keep the implementation simple. Manual testing also reinforced that local dev-server restarts can matter when validating fresh backend changes.</t>
   </si>
 </sst>
 </file>
@@ -1748,16 +1780,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E63"/>
-  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="19.899999999999999" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.26953125" defaultRowHeight="19.899999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="44.28515625" style="1" customWidth="1"/>
-    <col min="2" max="4" width="16.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="31.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="16.28515625" style="1"/>
+    <col min="1" max="1" width="44.26953125" style="1" customWidth="1"/>
+    <col min="2" max="4" width="16.26953125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31.453125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="16.26953125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.6" customHeight="1">
+    <row r="1" spans="1:5" ht="27.65" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1800,7 +1832,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="4" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
@@ -1817,7 +1849,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="5" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -1834,7 +1866,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="6" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>20</v>
       </c>
@@ -1851,7 +1883,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="7" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>24</v>
       </c>
@@ -1868,7 +1900,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="8" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>28</v>
       </c>
@@ -1885,7 +1917,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="9" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>32</v>
       </c>
@@ -1902,7 +1934,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="10" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A10" s="7" t="s">
         <v>36</v>
       </c>
@@ -1919,7 +1951,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="11" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A11" s="7" t="s">
         <v>40</v>
       </c>
@@ -1936,7 +1968,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="12" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A12" s="7" t="s">
         <v>44</v>
       </c>
@@ -1953,357 +1985,367 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="20.100000000000001" customHeight="1">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-    </row>
-    <row r="14" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="13" spans="1:5" ht="20.149999999999999" customHeight="1">
+      <c r="A13" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
     </row>
-    <row r="15" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="15" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
     </row>
-    <row r="16" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="16" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="17" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
     </row>
-    <row r="18" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="18" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
     </row>
-    <row r="19" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="19" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A19" s="7"/>
       <c r="B19" s="8"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
     </row>
-    <row r="20" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="20" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A20" s="7"/>
       <c r="B20" s="8"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
     </row>
-    <row r="21" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="21" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A21" s="7"/>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
     </row>
-    <row r="22" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="22" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="8"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
     </row>
-    <row r="23" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="23" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A23" s="10"/>
       <c r="B23" s="8"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
     </row>
-    <row r="24" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="24" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A24" s="7"/>
       <c r="B24" s="8"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
     </row>
-    <row r="25" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="25" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A25" s="7"/>
       <c r="B25" s="8"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
     </row>
-    <row r="26" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="26" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A26" s="7"/>
       <c r="B26" s="8"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
     </row>
-    <row r="27" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="27" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A27" s="7"/>
       <c r="B27" s="8"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
     </row>
-    <row r="28" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="28" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A28" s="7"/>
       <c r="B28" s="8"/>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
     </row>
-    <row r="29" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="29" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A29" s="7"/>
       <c r="B29" s="8"/>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
     </row>
-    <row r="30" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="30" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A30" s="7"/>
       <c r="B30" s="8"/>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
     </row>
-    <row r="31" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="31" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A31" s="7"/>
       <c r="B31" s="8"/>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
     </row>
-    <row r="32" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="32" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A32" s="7"/>
       <c r="B32" s="8"/>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
     </row>
-    <row r="33" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="33" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A33" s="7"/>
       <c r="B33" s="8"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="34" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A34" s="7"/>
       <c r="B34" s="8"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
     </row>
-    <row r="35" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="35" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A35" s="7"/>
       <c r="B35" s="8"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
     </row>
-    <row r="36" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="36" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A36" s="7"/>
       <c r="B36" s="8"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
     </row>
-    <row r="37" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="37" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A37" s="7"/>
       <c r="B37" s="8"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="38" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A38" s="7"/>
       <c r="B38" s="8"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
     </row>
-    <row r="39" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="39" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A39" s="7"/>
       <c r="B39" s="8"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
     </row>
-    <row r="40" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="40" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A40" s="7"/>
       <c r="B40" s="8"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
     </row>
-    <row r="41" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="41" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A41" s="7"/>
       <c r="B41" s="8"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="42" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A42" s="7"/>
       <c r="B42" s="8"/>
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
       <c r="E42" s="9"/>
     </row>
-    <row r="43" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="43" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A43" s="7"/>
       <c r="B43" s="8"/>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
       <c r="E43" s="9"/>
     </row>
-    <row r="44" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="44" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A44" s="7"/>
       <c r="B44" s="11"/>
       <c r="C44" s="9"/>
       <c r="D44" s="9"/>
       <c r="E44" s="9"/>
     </row>
-    <row r="45" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="45" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A45" s="10"/>
       <c r="B45" s="8"/>
       <c r="C45" s="9"/>
       <c r="D45" s="9"/>
       <c r="E45" s="9"/>
     </row>
-    <row r="46" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="46" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A46" s="10"/>
       <c r="B46" s="8"/>
       <c r="C46" s="9"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
     </row>
-    <row r="47" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="47" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A47" s="10"/>
       <c r="B47" s="8"/>
       <c r="C47" s="9"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
     </row>
-    <row r="48" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="48" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A48" s="10"/>
       <c r="B48" s="8"/>
       <c r="C48" s="9"/>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
     </row>
-    <row r="49" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="49" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A49" s="10"/>
       <c r="B49" s="8"/>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
     </row>
-    <row r="50" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="50" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A50" s="10"/>
       <c r="B50" s="8"/>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
     </row>
-    <row r="51" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="51" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A51" s="10"/>
       <c r="B51" s="8"/>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
     </row>
-    <row r="52" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="52" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A52" s="10"/>
       <c r="B52" s="8"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
     </row>
-    <row r="53" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="53" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A53" s="10"/>
       <c r="B53" s="8"/>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
     </row>
-    <row r="54" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="54" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A54" s="10"/>
       <c r="B54" s="8"/>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
     </row>
-    <row r="55" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="55" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A55" s="10"/>
       <c r="B55" s="8"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
     </row>
-    <row r="56" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="56" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A56" s="10"/>
       <c r="B56" s="8"/>
       <c r="C56" s="9"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
     </row>
-    <row r="57" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="57" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A57" s="10"/>
       <c r="B57" s="8"/>
       <c r="C57" s="9"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
     </row>
-    <row r="58" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="58" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A58" s="10"/>
       <c r="B58" s="8"/>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
     </row>
-    <row r="59" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="59" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A59" s="10"/>
       <c r="B59" s="8"/>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
     </row>
-    <row r="60" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="60" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A60" s="10"/>
       <c r="B60" s="8"/>
       <c r="C60" s="9"/>
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
     </row>
-    <row r="61" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="61" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A61" s="10"/>
       <c r="B61" s="8"/>
       <c r="C61" s="9"/>
       <c r="D61" s="9"/>
       <c r="E61" s="9"/>
     </row>
-    <row r="62" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="62" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A62" s="10"/>
       <c r="B62" s="8"/>
       <c r="C62" s="9"/>
       <c r="D62" s="9"/>
       <c r="E62" s="9"/>
     </row>
-    <row r="63" spans="1:5" ht="20.100000000000001" customHeight="1">
+    <row r="63" spans="1:5" ht="20.149999999999999" customHeight="1">
       <c r="A63" s="10"/>
       <c r="B63" s="8"/>
       <c r="C63" s="9"/>

</xml_diff>

<commit_message>
feat: add assessments backend read and update flow
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -910,9 +910,80 @@
         <v>This iteration worked well because the payload requirements were made explicit and the visual direction was tied to the already-working students page. That kept the slice small, coherent, and easy to validate. The next step should complete the classes frontend flow with edit/delete actions.</v>
       </c>
     </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str" xml:space="preserve">
+        <v xml:space="preserve"># Implementer Prompt - Iteration 13
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-13/00-iteration-brief.md
+- sistema/docs/iterations/iteration-13/01-planner-output.md
+- sistema/client/src/pages/ClassesPage.tsx
+- sistema/client/src/config/classesApi.ts
+- sistema/client/src/styles.css
+- sistema/client/src/types/domain.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</v>
+      </c>
+      <c r="B15" t="str">
+        <v>The implementation behaved correctly and completed the basic classes frontend flow, but the classes page now concentrates create, edit, and delete behavior in one component. The current localized approach still works, yet future iterations should keep guarding against excessive UI-state and stylesheet growth.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Good frontend iteration. The agent preserved the current visual style, added edit and delete cleanly, and kept the classes flow coherent without unnecessary complexity.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>This iteration worked well because the payload requirements were made explicit and the visual direction was tied to the already-working students page. That kept the slice small, coherent, and easy to validate. The next step should complete the classes frontend flow with edit/delete actions.</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str" xml:space="preserve">
+        <v xml:space="preserve"># Implementer Prompt - Iteration 14
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-14/00-iteration-brief.md
+- sistema/docs/iterations/iteration-14/01-planner-output.md
+- sistema/server/src/modules/assessments/index.ts
+- sistema/server/src/routes/index.ts
+- sistema/server/src/shared/types/domain.ts
+- sistema/server/src/modules/classes/class.repository.ts
+- sistema/server/data/classes.json
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</v>
+      </c>
+      <c r="B16" t="str">
+        <v>The implementation behaved correctly and stayed within scope, but successful manual validation required using a class with actual enrolled student ids. The persistence model is intentionally simple and the classes repository now holds a small amount of assessment-specific support logic.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Good backend iteration. The agent stayed disciplined, implemented the first useful assessments slice, and preserved a simple persistence model without overengineering.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>This iteration worked well because the scope was tightly limited to one read flow and one single-cell update flow. Requiring strict validation for class, student, goal, and concept kept the behavior predictable. The resulting structure is simple enough to support the future assessments UI without prematurely expanding into notifications or analytics.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add class student enrollment frontend flow
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -981,9 +981,45 @@
         <v>This iteration worked well because the scope was tightly limited to one read flow and one single-cell update flow. Requiring strict validation for class, student, goal, and concept kept the behavior predictable. The resulting structure is simple enough to support the future assessments UI without prematurely expanding into notifications or analytics.</v>
       </c>
     </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str" xml:space="preserve">
+        <v xml:space="preserve"># Implementer Prompt - Iteration 15
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-15/00-iteration-brief.md
+- sistema/docs/iterations/iteration-15/01-planner-output.md
+- sistema/client/src/pages/ClassesPage.tsx
+- sistema/client/src/config/classesApi.ts
+- sistema/client/src/config/studentsApi.ts
+- sistema/client/src/styles.css
+- sistema/client/src/types/domain.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</v>
+      </c>
+      <c r="B17" t="str">
+        <v>The implementation behaved correctly and completed the missing student enrollment flow, but the classes page now holds more local UI state and the shared stylesheet continues to grow. The current solution is still coherent and localized, but future iterations should keep avoiding excessive page-level complexity.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Good frontend iteration. The agent reused the existing students API cleanly, added enrollment without overengineering, and kept the classes page behavior consistent.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>This iteration worked well because the prompt explicitly forced reuse of the existing students API and asked for a simple checkbox-based enrollment flow. That kept the implementation small, predictable, and easy to validate. With this slice complete, the classes frontend now supports the enrolled-student flow needed before building the assessments UI.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: make assessments matrix usable for first launch
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1017,9 +1017,44 @@
         <v>This iteration worked well because the prompt explicitly forced reuse of the existing students API and asked for a simple checkbox-based enrollment flow. That kept the implementation small, predictable, and easy to validate. With this slice complete, the classes frontend now supports the enrolled-student flow needed before building the assessments UI.</v>
       </c>
     </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str" xml:space="preserve">
+        <v xml:space="preserve"># Implementer Prompt - Iteration 19
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-19/00-iteration-brief.md
+- sistema/docs/iterations/iteration-19/01-planner-output.md
+- sistema/client/src/pages/AssessmentsPage.tsx
+- sistema/client/src/config/assessmentsApi.ts
+- sistema/client/src/styles.css
+- sistema/client/src/types/domain.ts
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</v>
+      </c>
+      <c r="B18" t="str">
+        <v>The implementation behaved correctly and stayed within scope. The main tradeoffs are the additional state branching in the assessments page and the decision to hardcode the first-use goals (`Requirements`, `Tests`) in the frontend. This is acceptable for the experiment now, but could become a limitation only if later requirements demanded configurable goals.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Good corrective iteration. The agent fixed a real functional gap in the assessments workflow without over-expanding scope, and the page now behaves much more like a usable management screen.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>This iteration was important because it removed the dependence on preexisting stored goals in the backend just to make the assessments page usable. That makes the assessments workflow practically complete enough to support the next required feature: daily consolidated notifications by email.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add daily notifications backend and demo UI
</commit_message>
<xml_diff>
--- a/HistóricoDoMeuExperimento.xlsx
+++ b/HistóricoDoMeuExperimento.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1052,9 +1052,46 @@
         <v>This iteration was important because it removed the dependence on preexisting stored goals in the backend just to make the assessments page usable. That makes the assessments workflow practically complete enough to support the next required feature: daily consolidated notifications by email.</v>
       </c>
     </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str" xml:space="preserve">
+        <v xml:space="preserve"># Implementer Prompt - Iteration 20
+Before making any code changes, read and consider these files from the workspace:
+- sistema/.github/copilot-instructions.md
+- sistema/docs/project-scope.md
+- sistema/docs/iterations/iteration-20/00-iteration-brief.md
+- sistema/docs/iterations/iteration-20/01-planner-output.md
+- sistema/server/src/modules/notifications/index.ts
+- sistema/server/src/modules/assessments/index.ts
+- sistema/server/src/modules/assessments/assessment.service.ts
+- sistema/server/src/routes/index.ts
+- sistema/server/src/shared/types/domain.ts
+- sistema/server/data/README.md
+Do not edit any file yet.
+First, respond only with:
+1. Objective
+2. Files you intend to change
+3. Out of scope
+4. Short implementation plan
+5. Manual validation steps
+6. Risks or caveats
+Wait for my approval before making changes.</v>
+      </c>
+      <c r="B19" t="str">
+        <v>The implementation behaved correctly and stayed within scope. The main tradeoffs are that dispatch remains manually triggered and email delivery is still development-oriented for local/demo safety. The Notifications page also depends on combining notifications data with student/class data to display friendly labels.</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Accepted</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Very good iteration. The backend notifications requirement was implemented correctly, and the added visibility layer solved the demonstration gap without requiring a separate iteration.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>This iteration became stronger after the follow-up UI visibility layer was added. Without that page, notifications would only be visible through logs and JSON files. With the Notifications page in place, the feature is now both implemented and demonstrable in the running application.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>